<commit_message>
Fix malformed scan-range cells in MAY.xlsx
Corrects the 20 cells flagged in scan_log_issues.csv (transposed digits,
dropped commas, descending ranges), which were inventing hundreds of
phantom scan numbers and leaving real scans unmatched.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel_filer/MAY.xlsx
+++ b/excel_filer/MAY.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\madsl\article\Article_OCT_Diabetic_neuropathy\excel_filer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{305CFA04-1310-468A-98DF-33441C39AA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B523E8-B947-4FE9-B850-AF1A498D90C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA0DDF78-1E24-467F-846A-13E733A53AE0}"/>
   </bookViews>
@@ -255,9 +255,6 @@
     <t>1502-1506</t>
   </si>
   <si>
-    <t>1058-1513</t>
-  </si>
-  <si>
     <t>1522-1527</t>
   </si>
   <si>
@@ -453,9 +450,6 @@
     <t>1827-1831</t>
   </si>
   <si>
-    <t>1833-138</t>
-  </si>
-  <si>
     <t>1839-1841, 1843-1844</t>
   </si>
   <si>
@@ -630,18 +624,12 @@
     <t>2173-2177</t>
   </si>
   <si>
-    <t>2179-2484</t>
-  </si>
-  <si>
     <t>2189-2193</t>
   </si>
   <si>
     <t>2200-2204</t>
   </si>
   <si>
-    <t>5506-2211</t>
-  </si>
-  <si>
     <t>2214-2218</t>
   </si>
   <si>
@@ -693,9 +681,6 @@
     <t>2291-2295</t>
   </si>
   <si>
-    <t>2316-2312</t>
-  </si>
-  <si>
     <t>2329-2334</t>
   </si>
   <si>
@@ -750,9 +735,6 @@
     <t>2430-2434</t>
   </si>
   <si>
-    <t>2436-5441</t>
-  </si>
-  <si>
     <t>2417-2421</t>
   </si>
   <si>
@@ -951,9 +933,6 @@
     <t>2793-2798</t>
   </si>
   <si>
-    <t>2195-2160</t>
-  </si>
-  <si>
     <t>HP-41-DR</t>
   </si>
   <si>
@@ -1014,9 +993,6 @@
     <t>2963-2968</t>
   </si>
   <si>
-    <t>2955,29562959-2961</t>
-  </si>
-  <si>
     <t>2949-2954</t>
   </si>
   <si>
@@ -1137,9 +1113,6 @@
     <t>3093-3097</t>
   </si>
   <si>
-    <t>3099-3014</t>
-  </si>
-  <si>
     <t>3168-3172</t>
   </si>
   <si>
@@ -1194,9 +1167,6 @@
     <t>3272-3276</t>
   </si>
   <si>
-    <t>3278-32183</t>
-  </si>
-  <si>
     <t>3259-3263</t>
   </si>
   <si>
@@ -1281,9 +1251,6 @@
     <t>3421-3426</t>
   </si>
   <si>
-    <t>3427,2429-3432</t>
-  </si>
-  <si>
     <t>3434-3439</t>
   </si>
   <si>
@@ -1344,18 +1311,6 @@
     <t>3522-3526</t>
   </si>
   <si>
-    <t>3528-2533</t>
-  </si>
-  <si>
-    <t>2534-3538</t>
-  </si>
-  <si>
-    <t>2540-3545</t>
-  </si>
-  <si>
-    <t>3591-3959</t>
-  </si>
-  <si>
     <t>3597-3602</t>
   </si>
   <si>
@@ -1521,18 +1476,12 @@
     <t>3913-3918</t>
   </si>
   <si>
-    <t>2893-3897</t>
-  </si>
-  <si>
     <t>3899-3905</t>
   </si>
   <si>
     <t>3942-3947</t>
   </si>
   <si>
-    <t>3933-39343936,3938,3940</t>
-  </si>
-  <si>
     <t>3926-3931</t>
   </si>
   <si>
@@ -1557,9 +1506,6 @@
     <t>3988-3992</t>
   </si>
   <si>
-    <t>3994-2999</t>
-  </si>
-  <si>
     <t>3975-3979</t>
   </si>
   <si>
@@ -1623,9 +1569,6 @@
     <t>4152-4157</t>
   </si>
   <si>
-    <t>4134-4183</t>
-  </si>
-  <si>
     <t>4140-4145</t>
   </si>
   <si>
@@ -1663,6 +1606,63 @@
   </si>
   <si>
     <t>2160-2164</t>
+  </si>
+  <si>
+    <t>2179-2184</t>
+  </si>
+  <si>
+    <t>1508-1513</t>
+  </si>
+  <si>
+    <t>1833-1838</t>
+  </si>
+  <si>
+    <t>2312-2316</t>
+  </si>
+  <si>
+    <t>2436-2441</t>
+  </si>
+  <si>
+    <t>2955,2956,2959-2961</t>
+  </si>
+  <si>
+    <t>3099-3114</t>
+  </si>
+  <si>
+    <t>3278-3283</t>
+  </si>
+  <si>
+    <t>3427,3429-3432</t>
+  </si>
+  <si>
+    <t>3528-3533</t>
+  </si>
+  <si>
+    <t>3534-3538</t>
+  </si>
+  <si>
+    <t>3540-3545</t>
+  </si>
+  <si>
+    <t>3591-3595</t>
+  </si>
+  <si>
+    <t>3893-3897</t>
+  </si>
+  <si>
+    <t>3933-3934,3936,3938,3940</t>
+  </si>
+  <si>
+    <t>3994-3999</t>
+  </si>
+  <si>
+    <t>4134-4138</t>
+  </si>
+  <si>
+    <t>2195-2199</t>
+  </si>
+  <si>
+    <t>2200-2211</t>
   </si>
 </sst>
 </file>
@@ -2088,8 +2088,8 @@
   <dimension ref="A1:S68"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.42578125" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" customWidth="1"/>
     <col min="4" max="4" width="12.42578125" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
@@ -2153,22 +2153,22 @@
         <v>44335</v>
       </c>
       <c r="C2" t="s">
-        <v>542</v>
+        <v>523</v>
       </c>
       <c r="D2">
         <v>2165</v>
       </c>
       <c r="E2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="G2">
         <v>2178</v>
       </c>
       <c r="H2" t="s">
-        <v>198</v>
+        <v>524</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -2475,60 +2475,60 @@
         <v>1507</v>
       </c>
       <c r="K10" t="s">
-        <v>73</v>
+        <v>525</v>
       </c>
       <c r="L10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M10">
         <v>1521</v>
       </c>
       <c r="N10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" s="1">
         <v>44328</v>
       </c>
       <c r="C11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11">
         <v>1535</v>
       </c>
       <c r="E11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" t="s">
         <v>78</v>
-      </c>
-      <c r="F11" t="s">
-        <v>79</v>
       </c>
       <c r="G11">
         <v>1550</v>
       </c>
       <c r="H11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J11">
         <v>1543</v>
       </c>
       <c r="K11" t="s">
+        <v>87</v>
+      </c>
+      <c r="L11" t="s">
         <v>88</v>
-      </c>
-      <c r="L11" t="s">
-        <v>89</v>
       </c>
       <c r="M11">
         <v>1587</v>
       </c>
       <c r="N11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
@@ -2539,87 +2539,87 @@
         <v>44330</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D12">
         <v>1620</v>
       </c>
       <c r="E12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G12">
         <v>1633</v>
       </c>
       <c r="H12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J12">
         <v>1674</v>
       </c>
       <c r="K12" t="s">
+        <v>108</v>
+      </c>
+      <c r="L12" t="s">
         <v>109</v>
-      </c>
-      <c r="L12" t="s">
-        <v>110</v>
       </c>
       <c r="M12">
         <v>1686</v>
       </c>
       <c r="N12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="S12" t="s">
-        <v>541</v>
+        <v>522</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13" s="1">
         <v>44330</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D13">
         <v>1645</v>
       </c>
       <c r="E13" t="s">
+        <v>103</v>
+      </c>
+      <c r="F13" t="s">
         <v>104</v>
-      </c>
-      <c r="F13" t="s">
-        <v>105</v>
       </c>
       <c r="G13">
         <v>1657</v>
       </c>
       <c r="H13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J13">
         <v>1698</v>
       </c>
       <c r="K13" t="s">
+        <v>112</v>
+      </c>
+      <c r="L13" t="s">
         <v>113</v>
-      </c>
-      <c r="L13" t="s">
-        <v>114</v>
       </c>
       <c r="M13">
         <v>1711</v>
       </c>
       <c r="N13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -2630,294 +2630,294 @@
         <v>44330</v>
       </c>
       <c r="C14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D14">
         <v>1723</v>
       </c>
       <c r="E14" t="s">
+        <v>117</v>
+      </c>
+      <c r="F14" t="s">
         <v>118</v>
-      </c>
-      <c r="F14" t="s">
-        <v>119</v>
       </c>
       <c r="G14">
         <v>1735</v>
       </c>
       <c r="H14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J14">
         <v>1771</v>
       </c>
       <c r="K14" t="s">
+        <v>125</v>
+      </c>
+      <c r="L14" t="s">
         <v>126</v>
-      </c>
-      <c r="L14" t="s">
-        <v>127</v>
       </c>
       <c r="M14">
         <v>1784</v>
       </c>
       <c r="N14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B15" s="1">
         <v>44330</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D15">
         <v>1747</v>
       </c>
       <c r="E15" t="s">
+        <v>121</v>
+      </c>
+      <c r="F15" t="s">
         <v>122</v>
-      </c>
-      <c r="F15" t="s">
-        <v>123</v>
       </c>
       <c r="G15">
         <v>1759</v>
       </c>
       <c r="H15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J15">
         <v>1796</v>
       </c>
       <c r="K15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L15" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M15">
         <v>1808</v>
       </c>
       <c r="N15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B16" s="1">
         <v>44333</v>
       </c>
       <c r="C16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D16">
         <v>1832</v>
       </c>
       <c r="E16" t="s">
-        <v>139</v>
+        <v>526</v>
       </c>
       <c r="F16" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G16">
         <v>1845</v>
       </c>
       <c r="H16" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I16" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J16">
         <v>1890</v>
       </c>
       <c r="K16" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L16" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="M16">
         <v>1904</v>
       </c>
       <c r="N16" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B17" s="1">
         <v>44333</v>
       </c>
       <c r="C17" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D17">
         <v>1858</v>
       </c>
       <c r="E17" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F17" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G17">
         <v>1870</v>
       </c>
       <c r="H17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B18" s="1">
         <v>44333</v>
       </c>
       <c r="C18" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D18">
         <v>1916</v>
       </c>
       <c r="E18" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F18" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G18">
         <v>1930</v>
       </c>
       <c r="H18" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B19" s="1">
         <v>44333</v>
       </c>
       <c r="C19" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D19">
         <v>1947</v>
       </c>
       <c r="E19" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F19" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G19">
         <v>1959</v>
       </c>
       <c r="H19" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B20" s="1">
         <v>44334</v>
       </c>
       <c r="C20" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D20">
         <v>1986</v>
       </c>
       <c r="E20" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F20" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G20">
         <v>1999</v>
       </c>
       <c r="H20" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I20" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="J20">
         <v>2038</v>
       </c>
       <c r="K20" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="L20" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="M20">
         <v>205</v>
       </c>
       <c r="N20" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B21" s="1">
         <v>44334</v>
       </c>
       <c r="C21" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D21">
         <v>2011</v>
       </c>
       <c r="E21" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F21" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G21">
         <v>2025</v>
       </c>
       <c r="H21" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I21" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="J21">
         <v>2062</v>
       </c>
       <c r="K21" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="L21" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M21">
         <v>2074</v>
       </c>
       <c r="N21" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -2928,364 +2928,364 @@
         <v>44334</v>
       </c>
       <c r="C22" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D22">
         <v>2087</v>
       </c>
       <c r="E22" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F22" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G22">
         <v>2099</v>
       </c>
       <c r="H22" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I22" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="J22">
         <v>2119</v>
       </c>
       <c r="K22" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="L22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="M22">
         <v>2132</v>
       </c>
       <c r="N22" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B23" s="1">
         <v>44335</v>
       </c>
       <c r="C23" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D23">
         <v>2194</v>
       </c>
       <c r="E23" t="s">
-        <v>305</v>
+        <v>541</v>
       </c>
       <c r="F23" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G23">
         <v>2205</v>
       </c>
       <c r="H23" t="s">
-        <v>201</v>
+        <v>542</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B24" s="1">
         <v>44335</v>
       </c>
       <c r="C24" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D24">
         <v>2225</v>
       </c>
       <c r="E24" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="F24" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="G24">
         <v>2238</v>
       </c>
       <c r="H24" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B25" s="1">
         <v>44336</v>
       </c>
       <c r="C25" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D25">
         <v>2272</v>
       </c>
       <c r="E25" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F25" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="G25">
         <v>2284</v>
       </c>
       <c r="H25" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="I25" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="J25">
         <v>2328</v>
       </c>
       <c r="K25" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="L25" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="M25">
         <v>2340</v>
       </c>
       <c r="N25" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B26" s="1">
         <v>44336</v>
       </c>
       <c r="C26" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D26">
         <v>2296</v>
       </c>
       <c r="E26" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="F26" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="G26">
         <v>2315</v>
       </c>
       <c r="H26" t="s">
-        <v>219</v>
+        <v>527</v>
       </c>
       <c r="I26" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="J26">
         <v>2353</v>
       </c>
       <c r="K26" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="L26" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="M26">
         <v>2367</v>
       </c>
       <c r="N26" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B27" s="9">
         <v>44336</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="D27" s="10">
         <v>2380</v>
       </c>
       <c r="E27" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="F27" s="10" t="s">
         <v>230</v>
-      </c>
-      <c r="F27" s="10" t="s">
-        <v>235</v>
       </c>
       <c r="G27" s="10">
         <v>2392</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="J27" s="10">
         <v>2422</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="L27" s="10" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="M27" s="10">
         <v>2435</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>238</v>
+        <v>528</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B28" s="1">
         <v>44337</v>
       </c>
       <c r="C28" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="D28">
         <v>2449</v>
       </c>
       <c r="E28" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="F28" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="G28">
         <v>2462</v>
       </c>
       <c r="H28" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="I28" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="J28">
         <v>2483</v>
       </c>
       <c r="K28" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="L28" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="M28">
         <v>2495</v>
       </c>
       <c r="N28" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="B29" s="1">
         <v>44337</v>
       </c>
       <c r="C29" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="D29">
         <v>2518</v>
       </c>
       <c r="E29" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="F29" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="G29">
         <v>2530</v>
       </c>
       <c r="H29" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="B30" s="1">
         <v>44340</v>
       </c>
       <c r="C30" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="D30">
         <v>2544</v>
       </c>
       <c r="E30" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="F30" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="G30">
         <v>2557</v>
       </c>
       <c r="H30" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B31" s="1">
         <v>44340</v>
       </c>
       <c r="C31" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="D31">
         <v>2587</v>
       </c>
       <c r="E31" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="F31" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="G31">
         <v>2599</v>
       </c>
       <c r="H31" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="I31" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="J31">
         <v>2611</v>
       </c>
       <c r="K31" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="L31" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="M31">
         <v>2623</v>
       </c>
       <c r="N31" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -3296,1283 +3296,1283 @@
         <v>44340</v>
       </c>
       <c r="C32" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="D32">
         <v>2635</v>
       </c>
       <c r="E32" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="F32" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="G32">
         <v>2647</v>
       </c>
       <c r="H32" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="I32" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="J32">
         <v>2687</v>
       </c>
       <c r="K32" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="L32" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="M32">
         <v>2699</v>
       </c>
       <c r="N32" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B33" s="1">
         <v>44340</v>
       </c>
       <c r="C33" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="D33">
         <v>2660</v>
       </c>
       <c r="E33" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="F33" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="G33">
         <v>2675</v>
       </c>
       <c r="H33" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="I33" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="J33">
         <v>2712</v>
       </c>
       <c r="K33" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="L33" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="M33">
         <v>2728</v>
       </c>
       <c r="N33" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="B34" s="1">
         <v>44341</v>
       </c>
       <c r="C34" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D34">
         <v>2742</v>
       </c>
       <c r="E34" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="F34" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="G34">
         <v>2755</v>
       </c>
       <c r="H34" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="B35" s="1">
         <v>44341</v>
       </c>
       <c r="C35" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="D35">
         <v>2768</v>
       </c>
       <c r="E35" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="F35" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="G35">
         <v>2780</v>
       </c>
       <c r="H35" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="I35" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="J35">
         <v>2792</v>
       </c>
       <c r="K35" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="L35" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="M35">
         <v>2806</v>
       </c>
       <c r="N35" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="B36" s="1">
         <v>44341</v>
       </c>
       <c r="C36" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="D36">
         <v>2818</v>
       </c>
       <c r="E36" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
       <c r="F36" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="G36">
         <v>2831</v>
       </c>
       <c r="H36" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="B37" s="1">
         <v>44341</v>
       </c>
       <c r="C37" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="D37">
         <v>2853</v>
       </c>
       <c r="E37" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="F37" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="G37">
         <v>2866</v>
       </c>
       <c r="H37" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="B38" s="1">
         <v>44281</v>
       </c>
       <c r="C38" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="D38">
         <v>2900</v>
       </c>
       <c r="E38" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="F38" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="G38">
         <v>2912</v>
       </c>
       <c r="H38" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="B39" s="1">
         <v>44281</v>
       </c>
       <c r="C39" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="D39">
         <v>2924</v>
       </c>
       <c r="E39" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="F39" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="G39">
         <v>2936</v>
       </c>
       <c r="H39" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B40" s="1">
         <v>44281</v>
       </c>
       <c r="C40" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="D40">
         <v>2948</v>
       </c>
       <c r="E40" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="F40" t="s">
-        <v>326</v>
+        <v>529</v>
       </c>
       <c r="G40">
         <v>2962</v>
       </c>
       <c r="H40" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="I40" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="J40">
         <v>3000</v>
       </c>
       <c r="K40" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="L40" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="M40">
         <v>3013</v>
       </c>
       <c r="N40" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="B41" s="1">
         <v>44281</v>
       </c>
       <c r="C41" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="D41">
         <v>2974</v>
       </c>
       <c r="E41" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="F41" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="G41">
         <v>2987</v>
       </c>
       <c r="H41" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="B42" s="1">
         <v>44281</v>
       </c>
       <c r="C42" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="D42" t="s">
-        <v>539</v>
+        <v>520</v>
       </c>
       <c r="E42">
         <v>3031</v>
       </c>
       <c r="F42" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="G42">
         <v>3040</v>
       </c>
       <c r="H42" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="I42" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="J42">
         <v>3054</v>
       </c>
       <c r="K42" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="L42" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="M42">
         <v>3067</v>
       </c>
       <c r="N42" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B43" s="1">
         <v>44282</v>
       </c>
       <c r="C43" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="D43">
         <v>3098</v>
       </c>
       <c r="E43" t="s">
-        <v>367</v>
+        <v>530</v>
       </c>
       <c r="F43" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="G43">
         <v>3110</v>
       </c>
       <c r="H43" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="I43" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="J43">
         <v>3125</v>
       </c>
       <c r="K43" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="L43" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="M43">
         <v>3138</v>
       </c>
       <c r="N43" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="B44" s="1">
         <v>44282</v>
       </c>
       <c r="C44" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="D44">
         <v>3161</v>
       </c>
       <c r="E44" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="F44" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="G44">
         <v>3173</v>
       </c>
       <c r="H44" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
-        <v>540</v>
+        <v>521</v>
       </c>
       <c r="B45" s="1">
         <v>44282</v>
       </c>
       <c r="C45" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
       <c r="D45" s="3">
         <v>3185</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="F45" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="G45">
         <v>3198</v>
       </c>
       <c r="H45" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="B46" s="1">
         <v>44283</v>
       </c>
       <c r="C46" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="D46">
         <v>3264</v>
       </c>
       <c r="E46" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="F46" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="G46">
         <v>3277</v>
       </c>
       <c r="H46" t="s">
-        <v>386</v>
+        <v>531</v>
       </c>
       <c r="I46" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="J46">
         <v>3294</v>
       </c>
       <c r="K46" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="L46" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="M46">
         <v>3307</v>
       </c>
       <c r="N46" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="B47" s="1">
         <v>44283</v>
       </c>
       <c r="C47" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="D47" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="B48" s="1">
         <v>44283</v>
       </c>
       <c r="C48" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="D48">
         <v>3320</v>
       </c>
       <c r="E48" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
       <c r="F48" t="s">
-        <v>398</v>
+        <v>388</v>
       </c>
       <c r="G48">
         <v>3334</v>
       </c>
       <c r="H48" t="s">
-        <v>399</v>
+        <v>389</v>
       </c>
       <c r="I48" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="J48">
         <v>3371</v>
       </c>
       <c r="K48" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
       <c r="L48" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="M48">
         <v>3383</v>
       </c>
       <c r="N48" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
-        <v>395</v>
+        <v>385</v>
       </c>
       <c r="B49" s="1">
         <v>44283</v>
       </c>
       <c r="C49" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="D49">
         <v>3346</v>
       </c>
       <c r="E49" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="F49" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="G49">
         <v>3359</v>
       </c>
       <c r="H49" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="B50" s="1">
         <v>44283</v>
       </c>
       <c r="C50" t="s">
-        <v>411</v>
+        <v>401</v>
       </c>
       <c r="D50">
         <v>3396</v>
       </c>
       <c r="E50" t="s">
-        <v>412</v>
+        <v>402</v>
       </c>
       <c r="F50" t="s">
-        <v>409</v>
+        <v>399</v>
       </c>
       <c r="G50">
         <v>3408</v>
       </c>
       <c r="H50" t="s">
-        <v>410</v>
+        <v>400</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="B51" s="1">
         <v>44283</v>
       </c>
       <c r="C51" t="s">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="D51">
         <v>3420</v>
       </c>
       <c r="E51" t="s">
-        <v>414</v>
+        <v>404</v>
       </c>
       <c r="F51" t="s">
-        <v>415</v>
+        <v>532</v>
       </c>
       <c r="G51">
         <v>3433</v>
       </c>
       <c r="H51" t="s">
-        <v>416</v>
+        <v>405</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="B52" s="1">
         <v>44286</v>
       </c>
       <c r="C52" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="D52">
         <v>3447</v>
       </c>
       <c r="E52" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="F52" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="G52">
         <v>3460</v>
       </c>
       <c r="H52" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
       <c r="I52" t="s">
-        <v>429</v>
+        <v>418</v>
       </c>
       <c r="J52">
         <v>3502</v>
       </c>
       <c r="K52" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
       <c r="L52" t="s">
-        <v>427</v>
+        <v>416</v>
       </c>
       <c r="M52">
         <v>3515</v>
       </c>
       <c r="N52" t="s">
-        <v>428</v>
+        <v>417</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="B53" s="1">
         <v>44286</v>
       </c>
       <c r="C53" t="s">
-        <v>425</v>
+        <v>414</v>
       </c>
       <c r="D53">
         <v>3474</v>
       </c>
       <c r="E53" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
       <c r="F53" t="s">
-        <v>424</v>
+        <v>413</v>
       </c>
       <c r="G53">
         <v>3490</v>
       </c>
       <c r="H53" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="I53" t="s">
-        <v>435</v>
+        <v>424</v>
       </c>
       <c r="J53">
         <v>3527</v>
       </c>
       <c r="K53" t="s">
-        <v>436</v>
+        <v>533</v>
       </c>
       <c r="L53" t="s">
-        <v>437</v>
+        <v>534</v>
       </c>
       <c r="M53">
-        <v>2539</v>
+        <v>3539</v>
       </c>
       <c r="N53" t="s">
-        <v>438</v>
+        <v>535</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="B54" s="1">
         <v>44286</v>
       </c>
       <c r="C54" t="s">
-        <v>433</v>
+        <v>422</v>
       </c>
       <c r="D54">
         <v>3551</v>
       </c>
       <c r="E54" t="s">
-        <v>434</v>
+        <v>423</v>
       </c>
       <c r="F54" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
       <c r="G54">
         <v>3571</v>
       </c>
       <c r="H54" t="s">
-        <v>431</v>
+        <v>420</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="B55" s="1">
         <v>44286</v>
       </c>
       <c r="C55" t="s">
-        <v>441</v>
+        <v>426</v>
       </c>
       <c r="D55">
         <v>3583</v>
       </c>
       <c r="E55" t="s">
-        <v>442</v>
+        <v>427</v>
       </c>
       <c r="F55" t="s">
-        <v>439</v>
+        <v>536</v>
       </c>
       <c r="G55">
         <v>3596</v>
       </c>
       <c r="H55" t="s">
-        <v>440</v>
+        <v>425</v>
       </c>
       <c r="I55" t="s">
-        <v>445</v>
+        <v>430</v>
       </c>
       <c r="J55">
         <v>3608</v>
       </c>
       <c r="K55" t="s">
-        <v>446</v>
+        <v>431</v>
       </c>
       <c r="L55" t="s">
-        <v>443</v>
+        <v>428</v>
       </c>
       <c r="M55">
         <v>3620</v>
       </c>
       <c r="N55" t="s">
-        <v>444</v>
+        <v>429</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>447</v>
+        <v>432</v>
       </c>
       <c r="B56" s="1">
         <v>44348</v>
       </c>
       <c r="C56" t="s">
-        <v>450</v>
+        <v>435</v>
       </c>
       <c r="D56">
         <v>3633</v>
       </c>
       <c r="E56" t="s">
-        <v>451</v>
+        <v>436</v>
       </c>
       <c r="F56" t="s">
-        <v>448</v>
+        <v>433</v>
       </c>
       <c r="G56">
         <v>3647</v>
       </c>
       <c r="H56" t="s">
-        <v>449</v>
+        <v>434</v>
       </c>
       <c r="I56" t="s">
-        <v>456</v>
+        <v>441</v>
       </c>
       <c r="J56">
         <v>3669</v>
       </c>
       <c r="K56" t="s">
-        <v>457</v>
+        <v>442</v>
       </c>
       <c r="L56" t="s">
-        <v>454</v>
+        <v>439</v>
       </c>
       <c r="M56">
         <v>3681</v>
       </c>
       <c r="N56" t="s">
-        <v>455</v>
+        <v>440</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
-        <v>458</v>
+        <v>443</v>
       </c>
       <c r="B57" s="1">
         <v>44348</v>
       </c>
       <c r="C57" t="s">
-        <v>462</v>
+        <v>447</v>
       </c>
       <c r="D57">
         <v>3694</v>
       </c>
       <c r="E57" t="s">
-        <v>463</v>
+        <v>448</v>
       </c>
       <c r="F57" t="s">
-        <v>460</v>
+        <v>445</v>
       </c>
       <c r="G57">
         <v>3707</v>
       </c>
       <c r="H57" t="s">
-        <v>461</v>
+        <v>446</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
-        <v>459</v>
+        <v>444</v>
       </c>
       <c r="B58" s="1">
         <v>44348</v>
       </c>
       <c r="C58" t="s">
-        <v>466</v>
+        <v>451</v>
       </c>
       <c r="D58">
         <v>3719</v>
       </c>
       <c r="E58" t="s">
-        <v>467</v>
+        <v>452</v>
       </c>
       <c r="F58" t="s">
-        <v>464</v>
+        <v>449</v>
       </c>
       <c r="G58">
         <v>3731</v>
       </c>
       <c r="H58" t="s">
-        <v>465</v>
+        <v>450</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="B59" s="1">
         <v>44349</v>
       </c>
       <c r="C59" t="s">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="D59">
         <v>3744</v>
       </c>
       <c r="E59" t="s">
-        <v>471</v>
+        <v>456</v>
       </c>
       <c r="F59" t="s">
-        <v>470</v>
+        <v>455</v>
       </c>
       <c r="G59">
         <v>3759</v>
       </c>
       <c r="H59" t="s">
-        <v>469</v>
+        <v>454</v>
       </c>
       <c r="I59" t="s">
-        <v>479</v>
+        <v>464</v>
       </c>
       <c r="J59">
         <v>3798</v>
       </c>
       <c r="K59" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="L59" t="s">
-        <v>478</v>
+        <v>463</v>
       </c>
       <c r="M59">
         <v>3811</v>
       </c>
       <c r="N59" t="s">
-        <v>477</v>
+        <v>462</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
-        <v>447</v>
+        <v>432</v>
       </c>
       <c r="B60" s="1">
         <v>44349</v>
       </c>
       <c r="C60" t="s">
-        <v>476</v>
+        <v>461</v>
       </c>
       <c r="D60">
         <v>3772</v>
       </c>
       <c r="E60" t="s">
-        <v>475</v>
+        <v>460</v>
       </c>
       <c r="F60" t="s">
-        <v>474</v>
+        <v>459</v>
       </c>
       <c r="G60">
         <v>3786</v>
       </c>
       <c r="H60" t="s">
-        <v>473</v>
+        <v>458</v>
       </c>
       <c r="I60" t="s">
-        <v>484</v>
+        <v>469</v>
       </c>
       <c r="J60">
         <v>3824</v>
       </c>
       <c r="K60" t="s">
-        <v>483</v>
+        <v>468</v>
       </c>
       <c r="L60" t="s">
-        <v>482</v>
+        <v>467</v>
       </c>
       <c r="M60">
         <v>3837</v>
       </c>
       <c r="N60" t="s">
-        <v>481</v>
+        <v>466</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="B61" s="1">
         <v>44349</v>
       </c>
       <c r="C61" t="s">
-        <v>487</v>
+        <v>472</v>
       </c>
       <c r="D61">
         <v>3849</v>
       </c>
       <c r="E61" t="s">
-        <v>488</v>
+        <v>473</v>
       </c>
       <c r="F61" t="s">
-        <v>485</v>
+        <v>470</v>
       </c>
       <c r="G61">
         <v>3862</v>
       </c>
       <c r="H61" t="s">
-        <v>486</v>
+        <v>471</v>
       </c>
       <c r="I61" t="s">
-        <v>495</v>
+        <v>537</v>
       </c>
       <c r="J61">
         <v>3898</v>
       </c>
       <c r="K61" t="s">
-        <v>496</v>
+        <v>480</v>
       </c>
       <c r="L61" t="s">
-        <v>493</v>
+        <v>478</v>
       </c>
       <c r="M61">
         <v>3912</v>
       </c>
       <c r="N61" t="s">
-        <v>494</v>
+        <v>479</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
-        <v>468</v>
+        <v>453</v>
       </c>
       <c r="B62" s="1">
         <v>44349</v>
       </c>
       <c r="C62" t="s">
-        <v>491</v>
+        <v>476</v>
       </c>
       <c r="D62">
         <v>3874</v>
       </c>
       <c r="E62" t="s">
-        <v>492</v>
+        <v>477</v>
       </c>
       <c r="F62" t="s">
-        <v>489</v>
+        <v>474</v>
       </c>
       <c r="G62">
         <v>3886</v>
       </c>
       <c r="H62" t="s">
-        <v>490</v>
+        <v>475</v>
       </c>
       <c r="I62" t="s">
-        <v>500</v>
+        <v>483</v>
       </c>
       <c r="J62">
         <v>3935</v>
       </c>
       <c r="K62" t="s">
-        <v>499</v>
+        <v>482</v>
       </c>
       <c r="L62" t="s">
-        <v>498</v>
+        <v>538</v>
       </c>
       <c r="M62">
         <v>3941</v>
       </c>
       <c r="N62" t="s">
-        <v>497</v>
+        <v>481</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
-        <v>501</v>
+        <v>484</v>
       </c>
       <c r="B63" s="1">
         <v>44350</v>
       </c>
       <c r="C63" t="s">
-        <v>502</v>
+        <v>485</v>
       </c>
       <c r="D63">
         <v>3953</v>
       </c>
       <c r="E63" t="s">
-        <v>503</v>
+        <v>486</v>
       </c>
       <c r="F63" t="s">
-        <v>504</v>
+        <v>487</v>
       </c>
       <c r="G63">
         <v>3965</v>
       </c>
       <c r="H63" t="s">
-        <v>505</v>
+        <v>488</v>
       </c>
       <c r="I63" t="s">
-        <v>508</v>
+        <v>490</v>
       </c>
       <c r="J63">
         <v>3980</v>
       </c>
       <c r="K63" t="s">
-        <v>509</v>
+        <v>491</v>
       </c>
       <c r="L63" t="s">
-        <v>506</v>
+        <v>489</v>
       </c>
       <c r="M63">
         <v>3993</v>
       </c>
       <c r="N63" t="s">
-        <v>507</v>
+        <v>539</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
-        <v>510</v>
+        <v>492</v>
       </c>
       <c r="B64" s="1">
         <v>44350</v>
       </c>
       <c r="C64" t="s">
-        <v>513</v>
+        <v>495</v>
       </c>
       <c r="D64">
         <v>4006</v>
       </c>
       <c r="E64" t="s">
-        <v>514</v>
+        <v>496</v>
       </c>
       <c r="F64" t="s">
-        <v>511</v>
+        <v>493</v>
       </c>
       <c r="G64">
         <v>4018</v>
       </c>
       <c r="H64" t="s">
-        <v>512</v>
+        <v>494</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>468</v>
+        <v>453</v>
       </c>
       <c r="B65" s="1">
         <v>44350</v>
       </c>
       <c r="C65" t="s">
-        <v>515</v>
+        <v>497</v>
       </c>
       <c r="D65">
         <v>4040</v>
       </c>
       <c r="E65" t="s">
-        <v>516</v>
+        <v>498</v>
       </c>
       <c r="F65" t="s">
-        <v>518</v>
+        <v>500</v>
       </c>
       <c r="G65">
         <v>4052</v>
       </c>
       <c r="H65" t="s">
-        <v>517</v>
+        <v>499</v>
       </c>
       <c r="I65" t="s">
-        <v>521</v>
+        <v>503</v>
       </c>
       <c r="J65">
         <v>4087</v>
       </c>
       <c r="K65" t="s">
-        <v>522</v>
+        <v>504</v>
       </c>
       <c r="L65" t="s">
-        <v>520</v>
+        <v>502</v>
       </c>
       <c r="M65">
         <v>4103</v>
       </c>
       <c r="N65" t="s">
-        <v>519</v>
+        <v>501</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>501</v>
+        <v>484</v>
       </c>
       <c r="B66" s="1">
         <v>44351</v>
       </c>
       <c r="C66" t="s">
-        <v>525</v>
+        <v>507</v>
       </c>
       <c r="D66">
         <v>4114</v>
       </c>
       <c r="E66" t="s">
-        <v>526</v>
+        <v>508</v>
       </c>
       <c r="F66" t="s">
-        <v>523</v>
+        <v>505</v>
       </c>
       <c r="G66">
         <v>4127</v>
       </c>
       <c r="H66" t="s">
-        <v>524</v>
+        <v>506</v>
       </c>
       <c r="I66" t="s">
-        <v>533</v>
+        <v>514</v>
       </c>
       <c r="J66">
         <v>4166</v>
       </c>
       <c r="K66" t="s">
-        <v>534</v>
+        <v>515</v>
       </c>
       <c r="L66" t="s">
-        <v>532</v>
+        <v>513</v>
       </c>
       <c r="M66">
         <v>4178</v>
       </c>
       <c r="N66" t="s">
-        <v>531</v>
+        <v>512</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="B67" s="1">
         <v>44351</v>
       </c>
       <c r="C67" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="D67">
         <v>4139</v>
       </c>
       <c r="E67" t="s">
-        <v>530</v>
+        <v>511</v>
       </c>
       <c r="F67" t="s">
-        <v>527</v>
+        <v>509</v>
       </c>
       <c r="G67">
         <v>4151</v>
       </c>
       <c r="H67" t="s">
-        <v>528</v>
+        <v>510</v>
       </c>
       <c r="I67" t="s">
-        <v>537</v>
+        <v>518</v>
       </c>
       <c r="J67">
         <v>4191</v>
       </c>
       <c r="K67" t="s">
-        <v>536</v>
+        <v>517</v>
       </c>
       <c r="L67" t="s">
-        <v>538</v>
+        <v>519</v>
       </c>
       <c r="M67">
         <v>4206</v>
       </c>
       <c r="N67" t="s">
-        <v>535</v>
+        <v>516</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
@@ -4605,7 +4605,7 @@
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.25">
@@ -4613,7 +4613,7 @@
         <v>44328.447916666664</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D3" s="2">
         <v>44328.65625</v>
@@ -4696,190 +4696,190 @@
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="H4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="I4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="L4" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="N4" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="O4" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="P4" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="R4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="S4" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="T4" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="V4" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="W4" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="X4" t="s">
+        <v>344</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>345</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>349</v>
+      </c>
+      <c r="AA4" t="s">
         <v>352</v>
       </c>
-      <c r="Y4" t="s">
-        <v>353</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>357</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>360</v>
-      </c>
       <c r="AB4" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="AC4" t="s">
-        <v>453</v>
+        <v>438</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="M5" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="P5" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="R5" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="U5" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="AB5" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="AC5" t="s">
-        <v>452</v>
+        <v>437</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N6" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="P6" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="Q6" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="V6" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="Y6" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="AB6" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="J7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O7" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="P7" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="S7" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="T7" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="V7" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="W7" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="Z7" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="AA7" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -4897,12 +4897,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002B3BCDED8CEB614F82D24B72167991C4" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f2645664536588993a844ffd1bdf7759">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="2c543aac-2840-490e-b44c-daae2b99db87" xmlns:ns4="a33e0d94-a79c-488e-9710-b30b07881363" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b8379f2bd97f399b85d3d553c35997a6" ns3:_="" ns4:_="">
     <xsd:import namespace="2c543aac-2840-490e-b44c-daae2b99db87"/>
@@ -5125,6 +5119,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF1F42CA-1352-4137-B2EA-9A0759ADA840}">
   <ds:schemaRefs>
@@ -5134,23 +5134,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{267B2119-A360-4C94-B91A-7419872C01E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="2c543aac-2840-490e-b44c-daae2b99db87"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="a33e0d94-a79c-488e-9710-b30b07881363"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BE5A1A68-E502-4369-8117-1C5AD6114620}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5167,4 +5150,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{267B2119-A360-4C94-B91A-7419872C01E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="2c543aac-2840-490e-b44c-daae2b99db87"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="a33e0d94-a79c-488e-9710-b30b07881363"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>